<commit_message>
Update order flow system, config, and data cache - 2026-05-30
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-05.xlsx
+++ b/data/nifty_options/nifty_options_2026-05.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -905,6 +905,240 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>10:00:27</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>24343</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>16.76</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>-1.54</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24343.00 above TC 24279.70 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24343.00 above TC 24279.70 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>10:00:34</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>24198.2</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>17.18</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24198.20 below BC 24383.05 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD5" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24198.20 below BC 24383.05 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add gap ORB monitor, VWAP backtests, update order flow and data cache - 2026-05-30
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-05.xlsx
+++ b/data/nifty_options/nifty_options_2026-05.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1139,6 +1139,240 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>10:00:38</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>23874.85</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>18.74</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23874.85 below BC 24190.22 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD6" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23874.85 below BC 24190.22 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>10:00:35</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>23628.1</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>18.91</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23628.10 below BC 23898.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD7" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23628.10 below BC 23898.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add flag monitor, sector backtests, fix watchdog staleness check - 2026-06-01
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-05.xlsx
+++ b/data/nifty_options/nifty_options_2026-05.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1373,6 +1373,357 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>10:00:24</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>23369.4</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>19.87</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23369.40 below BC 23552.97 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD8" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23369.40 below BC 23552.97 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>10:00:40</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>23347.2</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23347.20 below BC 23724.80 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23347.20 below BC 23724.80 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>10:00:54</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>23679.25</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>18.97</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23679.25 above TC 23602.09 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD10" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23679.25 above TC 23602.09 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>